<commit_message>
used func like vlookup(), hlookup(), index matching and xlookup()
</commit_message>
<xml_diff>
--- a/EXCEL/Lookups.xlsx
+++ b/EXCEL/Lookups.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{5385FAB8-444E-46A4-9A1E-764B55F30D67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E3E7CD9F-3041-49AB-8208-5FFD646CD08B}"/>
+  <xr:revisionPtr revIDLastSave="76" documentId="13_ncr:1_{5385FAB8-444E-46A4-9A1E-764B55F30D67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF53B024-05DE-41E8-90D0-1AE31623605B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{86C2143A-C104-4631-B0C3-FAE18B7B60CC}"/>
+    <workbookView minimized="1" xWindow="2124" yWindow="2124" windowWidth="17280" windowHeight="10500" xr2:uid="{86C2143A-C104-4631-B0C3-FAE18B7B60CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Employees" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
   <si>
     <t>EmpID</t>
   </si>
@@ -89,7 +89,31 @@
     <t>Pune</t>
   </si>
   <si>
-    <t>v lookup</t>
+    <t>v lookup/ what is the dept of raj</t>
+  </si>
+  <si>
+    <t>dept</t>
+  </si>
+  <si>
+    <t>avg</t>
+  </si>
+  <si>
+    <t>it</t>
+  </si>
+  <si>
+    <t>hr</t>
+  </si>
+  <si>
+    <t>sc</t>
+  </si>
+  <si>
+    <t>avg salary of it guy</t>
+  </si>
+  <si>
+    <t>index match to get exact  salary</t>
+  </si>
+  <si>
+    <t>xlookup</t>
   </si>
 </sst>
 </file>
@@ -133,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -144,6 +168,11 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -159,6 +188,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -478,13 +511,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{818E6F0C-D68F-4B21-87C7-F723C2AF8CEA}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
+    <col min="1" max="1" width="10.7109375" customWidth="1"/>
     <col min="3" max="3" width="8.78515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.35546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="42" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" ht="84" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -503,8 +538,14 @@
       <c r="F1" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>101</v>
       </c>
@@ -524,8 +565,16 @@
         <f>VLOOKUP(A4,A1:E6,4,)</f>
         <v>55000</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G2">
+        <f>INDEX(D2:D6,MATCH(A4,A2:A6,0))</f>
+        <v>55000</v>
+      </c>
+      <c r="H2" t="str">
+        <f>_xlfn.XLOOKUP(A2,A2:A6,E2:E6,"not found")</f>
+        <v>Delhi</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>102</v>
       </c>
@@ -545,8 +594,16 @@
         <f t="shared" ref="F3:F6" si="0">VLOOKUP(A5,A2:E7,4,)</f>
         <v>80000</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G3">
+        <f t="shared" ref="G3:G6" si="1">INDEX(D3:D7,MATCH(A5,A3:A7,0))</f>
+        <v>80000</v>
+      </c>
+      <c r="H3" t="str">
+        <f t="shared" ref="H3:H6" si="2">_xlfn.XLOOKUP(A3,A3:A7,E3:E7,"not found")</f>
+        <v>Mumbai</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>103</v>
       </c>
@@ -566,8 +623,16 @@
         <f>VLOOKUP(A6,A3:E8,4,)</f>
         <v>50000</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G4">
+        <f t="shared" si="1"/>
+        <v>50000</v>
+      </c>
+      <c r="H4" t="str">
+        <f t="shared" si="2"/>
+        <v>Bangalore</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>104</v>
       </c>
@@ -587,8 +652,16 @@
         <f>VLOOKUP(A7,A4:E9,4,)</f>
         <v>#N/A</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G5" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="H5" t="str">
+        <f t="shared" si="2"/>
+        <v>Pune</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>105</v>
       </c>
@@ -607,6 +680,51 @@
       <c r="F6" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
+      </c>
+      <c r="G6" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="H6" t="str">
+        <f t="shared" si="2"/>
+        <v>Delhi</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11">
+        <v>80000</v>
+      </c>
+      <c r="C11">
+        <v>65000</v>
+      </c>
+      <c r="D11">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="42" x14ac:dyDescent="0.4">
+      <c r="A13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="6">
+        <f>HLOOKUP(B10,A10:D11,2)</f>
+        <v>80000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
use of sort, filter and randarray()
</commit_message>
<xml_diff>
--- a/EXCEL/Lookups.xlsx
+++ b/EXCEL/Lookups.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="13_ncr:1_{5385FAB8-444E-46A4-9A1E-764B55F30D67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF53B024-05DE-41E8-90D0-1AE31623605B}"/>
+  <xr:revisionPtr revIDLastSave="121" documentId="13_ncr:1_{5385FAB8-444E-46A4-9A1E-764B55F30D67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{809A9B28-544D-493D-80F6-BA7C4EF60324}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="2124" yWindow="2124" windowWidth="17280" windowHeight="10500" xr2:uid="{86C2143A-C104-4631-B0C3-FAE18B7B60CC}"/>
   </bookViews>
@@ -35,8 +35,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
   <si>
     <t>EmpID</t>
   </si>
@@ -114,6 +136,21 @@
   </si>
   <si>
     <t>xlookup</t>
+  </si>
+  <si>
+    <t>filter</t>
+  </si>
+  <si>
+    <t>sort</t>
+  </si>
+  <si>
+    <t>unique</t>
+  </si>
+  <si>
+    <t>random array</t>
+  </si>
+  <si>
+    <t>sort the it guy on the basis of salary</t>
   </si>
 </sst>
 </file>
@@ -145,7 +182,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -153,11 +190,143 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -168,11 +337,26 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -511,7 +695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{818E6F0C-D68F-4B21-87C7-F723C2AF8CEA}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
@@ -519,7 +703,7 @@
     <col min="6" max="6" width="9.35546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="84" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" ht="84" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -544,8 +728,11 @@
       <c r="H1" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="I1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>101</v>
       </c>
@@ -573,8 +760,12 @@
         <f>_xlfn.XLOOKUP(A2,A2:A6,E2:E6,"not found")</f>
         <v>Delhi</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="I2" cm="1">
+        <f t="array" aca="1" ref="I2:I6" ca="1">_xlfn.RANDARRAY(5,1,10000,50000)</f>
+        <v>40637.878985535797</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>102</v>
       </c>
@@ -602,8 +793,12 @@
         <f t="shared" ref="H3:H6" si="2">_xlfn.XLOOKUP(A3,A3:A7,E3:E7,"not found")</f>
         <v>Mumbai</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="I3">
+        <f ca="1"/>
+        <v>34018.691865127454</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>103</v>
       </c>
@@ -631,8 +826,12 @@
         <f t="shared" si="2"/>
         <v>Bangalore</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="I4">
+        <f ca="1"/>
+        <v>22250.097591367921</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>104</v>
       </c>
@@ -660,8 +859,12 @@
         <f t="shared" si="2"/>
         <v>Pune</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="I5">
+        <f ca="1"/>
+        <v>17453.509264509587</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>105</v>
       </c>
@@ -689,42 +892,277 @@
         <f t="shared" si="2"/>
         <v>Delhi</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A10" s="4" t="s">
+      <c r="I6">
+        <f ca="1"/>
+        <v>47908.222443703846</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A10" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="10" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A11" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="5">
         <v>80000</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="5">
         <v>65000</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="12">
         <v>50000</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="42" x14ac:dyDescent="0.4">
-      <c r="A13" s="5" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A12" s="11"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="12"/>
+    </row>
+    <row r="13" spans="1:9" ht="42" x14ac:dyDescent="0.4">
+      <c r="A13" s="13" t="s">
         <v>23</v>
       </c>
       <c r="B13" s="6">
         <f>HLOOKUP(B10,A10:D11,2)</f>
         <v>80000</v>
+      </c>
+      <c r="C13" s="7"/>
+      <c r="D13" s="14"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A16" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A17" s="16" cm="1">
+        <f t="array" ref="A17:H18">_xlfn._xlws.FILTER(A2:H6,C2:C6="IT","no emp found")</f>
+        <v>102</v>
+      </c>
+      <c r="B17" s="16" t="str">
+        <v>Raj</v>
+      </c>
+      <c r="C17" s="16" t="str">
+        <v>IT</v>
+      </c>
+      <c r="D17" s="16">
+        <v>65000</v>
+      </c>
+      <c r="E17" s="16" t="str">
+        <v>Mumbai</v>
+      </c>
+      <c r="F17" s="16">
+        <v>80000</v>
+      </c>
+      <c r="G17" s="16">
+        <v>80000</v>
+      </c>
+      <c r="H17" s="16" t="str">
+        <v>Mumbai</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A18" s="16">
+        <v>104</v>
+      </c>
+      <c r="B18" s="16" t="str">
+        <v>Karan</v>
+      </c>
+      <c r="C18" s="16" t="str">
+        <v>IT</v>
+      </c>
+      <c r="D18" s="16">
+        <v>80000</v>
+      </c>
+      <c r="E18" s="16" t="str">
+        <v>Pune</v>
+      </c>
+      <c r="F18" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G18" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H18" s="16" t="str">
+        <v>Pune</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A20" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A21" s="16" cm="1">
+        <f t="array" ref="A21:E25">_xlfn._xlws.SORT(A2:E6,4,-1)</f>
+        <v>104</v>
+      </c>
+      <c r="B21" s="16" t="str">
+        <v>Karan</v>
+      </c>
+      <c r="C21" s="16" t="str">
+        <v>IT</v>
+      </c>
+      <c r="D21" s="16">
+        <v>80000</v>
+      </c>
+      <c r="E21" s="16" t="str">
+        <v>Pune</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A22" s="16">
+        <v>102</v>
+      </c>
+      <c r="B22" s="16" t="str">
+        <v>Raj</v>
+      </c>
+      <c r="C22" s="16" t="str">
+        <v>IT</v>
+      </c>
+      <c r="D22" s="16">
+        <v>65000</v>
+      </c>
+      <c r="E22" s="16" t="str">
+        <v>Mumbai</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A23" s="16">
+        <v>103</v>
+      </c>
+      <c r="B23" s="16" t="str">
+        <v>Meena</v>
+      </c>
+      <c r="C23" s="16" t="str">
+        <v>Finance</v>
+      </c>
+      <c r="D23" s="16">
+        <v>55000</v>
+      </c>
+      <c r="E23" s="16" t="str">
+        <v>Bangalore</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A24" s="16">
+        <v>105</v>
+      </c>
+      <c r="B24" s="16" t="str">
+        <v>Sonia</v>
+      </c>
+      <c r="C24" s="16" t="str">
+        <v>HR</v>
+      </c>
+      <c r="D24" s="16">
+        <v>50000</v>
+      </c>
+      <c r="E24" s="16" t="str">
+        <v>Delhi</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A25" s="16">
+        <v>101</v>
+      </c>
+      <c r="B25" s="16" t="str">
+        <v>Aditi</v>
+      </c>
+      <c r="C25" s="16" t="str">
+        <v>HR</v>
+      </c>
+      <c r="D25" s="16">
+        <v>40000</v>
+      </c>
+      <c r="E25" s="16" t="str">
+        <v>Delhi</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A27" s="18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A28" s="19" t="str" cm="1">
+        <f t="array" ref="A28:A30">_xlfn.UNIQUE(C2:C6)</f>
+        <v>HR</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A29" s="19" t="str">
+        <v>IT</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A30" s="17" t="str">
+        <v>Finance</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="84" x14ac:dyDescent="0.4">
+      <c r="A32" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A33" cm="1">
+        <f t="array" ref="A33:E34">_xlfn._xlws.SORT(_xlfn._xlws.FILTER(A2:E6,C2:C6="IT"),4,-1)</f>
+        <v>104</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Karan</v>
+      </c>
+      <c r="C33" t="str">
+        <v>IT</v>
+      </c>
+      <c r="D33">
+        <v>80000</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Pune</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A34">
+        <v>102</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Raj</v>
+      </c>
+      <c r="C34" t="str">
+        <v>IT</v>
+      </c>
+      <c r="D34">
+        <v>65000</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Mumbai</v>
       </c>
     </row>
   </sheetData>

</xml_diff>